<commit_message>
feat(accel): unify Completed and Failed into Processed_Logs with auto-resolve retry flow
</commit_message>
<xml_diff>
--- a/projects/auto_page/autopageMKII/assets/tables/Accel_mode15-07-2026.xlsx
+++ b/projects/auto_page/autopageMKII/assets/tables/Accel_mode15-07-2026.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Failed_Orders" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Completed_Orders" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="แผ่นงาน5" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Processed_Logs" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -634,180 +635,20 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
           <t>0ZGDHNBL600035</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
-      <c r="Y2" t="inlineStr"/>
-      <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr"/>
-      <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="inlineStr"/>
-      <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr"/>
-      <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr"/>
-      <c r="AK2" t="inlineStr"/>
-      <c r="AL2" t="inlineStr"/>
-      <c r="AM2" t="inlineStr"/>
-      <c r="AN2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr"/>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr"/>
-      <c r="Y3" t="inlineStr"/>
-      <c r="Z3" t="inlineStr"/>
-      <c r="AA3" t="inlineStr"/>
-      <c r="AB3" t="inlineStr"/>
-      <c r="AC3" t="inlineStr"/>
-      <c r="AD3" t="inlineStr"/>
-      <c r="AE3" t="inlineStr"/>
-      <c r="AF3" t="inlineStr"/>
-      <c r="AG3" t="inlineStr"/>
-      <c r="AH3" t="inlineStr"/>
-      <c r="AI3" t="inlineStr"/>
-      <c r="AJ3" t="inlineStr"/>
-      <c r="AK3" t="inlineStr"/>
-      <c r="AL3" t="inlineStr"/>
-      <c r="AM3" t="inlineStr"/>
-      <c r="AN3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr"/>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
-      <c r="Y4" t="inlineStr"/>
-      <c r="Z4" t="inlineStr"/>
-      <c r="AA4" t="inlineStr"/>
-      <c r="AB4" t="inlineStr"/>
-      <c r="AC4" t="inlineStr"/>
-      <c r="AD4" t="inlineStr"/>
-      <c r="AE4" t="inlineStr"/>
-      <c r="AF4" t="inlineStr"/>
-      <c r="AG4" t="inlineStr"/>
-      <c r="AH4" t="inlineStr"/>
-      <c r="AI4" t="inlineStr"/>
-      <c r="AJ4" t="inlineStr"/>
-      <c r="AK4" t="inlineStr"/>
-      <c r="AL4" t="inlineStr"/>
-      <c r="AM4" t="inlineStr"/>
-      <c r="AN4" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="3"/>
+    <row r="4"/>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr"/>
-      <c r="X5" t="inlineStr"/>
-      <c r="Y5" t="inlineStr"/>
-      <c r="Z5" t="inlineStr"/>
-      <c r="AA5" t="inlineStr"/>
       <c r="AB5" t="inlineStr">
         <is>
           <t>W4LMTF087928</t>
         </is>
       </c>
-      <c r="AC5" t="inlineStr"/>
-      <c r="AD5" t="inlineStr"/>
-      <c r="AE5" t="inlineStr"/>
-      <c r="AF5" t="inlineStr"/>
-      <c r="AG5" t="inlineStr"/>
-      <c r="AH5" t="inlineStr"/>
-      <c r="AI5" t="inlineStr"/>
-      <c r="AJ5" t="inlineStr"/>
-      <c r="AK5" t="inlineStr"/>
-      <c r="AL5" t="inlineStr"/>
-      <c r="AM5" t="inlineStr"/>
-      <c r="AN5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1980,14 +1821,11 @@
           <t>B0183-W06-2607150006</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2010,14 +1848,11 @@
           <t>B0183-W06-2607150007</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2040,14 +1875,11 @@
           <t>B0183-W06-2607150008</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2070,14 +1902,11 @@
           <t>B0183-W06-2607150009</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2100,14 +1929,11 @@
           <t>B0183-W06-2607150010</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2130,14 +1956,11 @@
           <t>B0183-W06-2607150011</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2160,14 +1983,11 @@
           <t>B0183-W06-2607150012</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2190,14 +2010,11 @@
           <t>B0183-W06-2607150013</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2220,14 +2037,11 @@
           <t>B0183-W06-2607150014</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2250,14 +2064,11 @@
           <t>B0183-W06-2607150015</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2280,14 +2091,11 @@
           <t>B0183-W06-2607150016</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2310,14 +2118,11 @@
           <t>B0183-W06-2607150017</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2340,14 +2145,11 @@
           <t>B0183-W06-2607150018</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2370,14 +2172,11 @@
           <t>B0183-W06-2607150019</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2400,14 +2199,11 @@
           <t>B0183-W06-2607150020</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2430,14 +2226,11 @@
           <t>B0183-W06-2607150021</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2460,14 +2253,11 @@
           <t>B0183-W06-2607150022</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2490,14 +2280,11 @@
           <t>B0183-W06-2607150023</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2520,14 +2307,11 @@
           <t>B0183-W06-2607150024</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2550,14 +2334,11 @@
           <t>B0183-W06-2607150025</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2580,14 +2361,11 @@
           <t>B0183-W06-2607150026</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2610,14 +2388,11 @@
           <t>B0183-W06-2607150027</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2640,14 +2415,11 @@
           <t>B0183-W06-2607150028</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2670,14 +2442,11 @@
           <t>B0183-W06-2607150029</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2700,14 +2469,11 @@
           <t>B0183-W06-2607150030</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2730,14 +2496,11 @@
           <t>B0183-W06-2607150031</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2760,14 +2523,11 @@
           <t>B0183-W06-2607150032</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2790,14 +2550,11 @@
           <t>B0183-W06-2607150033</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2820,14 +2577,11 @@
           <t>B0183-W06-2607150034</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2850,14 +2604,11 @@
           <t>B0183-W06-2607150035</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2880,14 +2631,11 @@
           <t>B0183-W06-2607150036</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2910,14 +2658,11 @@
           <t>B0183-W06-2607150037</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2940,14 +2685,11 @@
           <t>B0183-W06-2607150038</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2970,14 +2712,11 @@
           <t>B0183-W06-2607150039</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3000,14 +2739,11 @@
           <t>B0183-W06-2607150040</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3030,14 +2766,11 @@
           <t>B0183-W06-2607150041</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3060,14 +2793,11 @@
           <t>B0183-W06-2607150042</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3090,14 +2820,11 @@
           <t>B0183-W06-2607150043</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3120,14 +2847,11 @@
           <t>B0183-W06-2607150044</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3150,14 +2874,11 @@
           <t>B0183-W06-2607150045</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3180,14 +2901,11 @@
           <t>B0183-W06-2607150046</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3210,14 +2928,11 @@
           <t>B0183-W06-2607150047</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr"/>
-      <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -3240,14 +2955,11 @@
           <t>B0183-W06-2607150048</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
-      <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3270,14 +2982,11 @@
           <t>B0183-W06-2607150049</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr"/>
-      <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3300,14 +3009,11 @@
           <t>B0183-W06-2607150050</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
-      <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3330,14 +3036,11 @@
           <t>B0183-W06-2607150051</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
-      <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3360,14 +3063,11 @@
           <t>B0183-W06-2607150052</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
-      <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3390,14 +3090,11 @@
           <t>B0183-W06-2607150053</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr"/>
-      <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3420,14 +3117,11 @@
           <t>B0183-W06-2607150054</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr"/>
-      <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3450,14 +3144,11 @@
           <t>B0183-W06-2607150055</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr"/>
-      <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3480,14 +3171,11 @@
           <t>B0183-W06-2607150056</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr"/>
-      <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3510,14 +3198,11 @@
           <t>B0183-W06-2607150057</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr"/>
-      <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3540,14 +3225,11 @@
           <t>B0183-W06-2607150058</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr"/>
-      <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3570,14 +3252,11 @@
           <t>B0183-W06-2607150059</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr"/>
-      <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3600,14 +3279,11 @@
           <t>B0183-W06-2607150060</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr"/>
-      <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3630,14 +3306,11 @@
           <t>B0183-W06-2607150061</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr"/>
-      <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3660,14 +3333,11 @@
           <t>B0183-W06-2607150062</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr"/>
-      <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3690,14 +3360,11 @@
           <t>B0183-W06-2607150063</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr"/>
-      <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3720,14 +3387,11 @@
           <t>B0183-W06-2607150064</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr"/>
-      <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3735,21 +3399,16 @@
           <t>2026-07-15 16:57:00</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr">
         <is>
           <t>260714N1AW2J8A</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr"/>
-      <c r="E61" t="inlineStr"/>
-      <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
           <t>ข้าม (สถานะ: ยกเลิกแล้ว)</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3772,14 +3431,11 @@
           <t>B0183-W06-2607150065</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr"/>
-      <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3802,14 +3458,11 @@
           <t>B0183-W06-2607150066</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr"/>
-      <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3832,14 +3485,11 @@
           <t>B0183-W06-2607150067</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr"/>
-      <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3862,14 +3512,11 @@
           <t>B0183-W06-2607150068</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr"/>
-      <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3892,14 +3539,11 @@
           <t>B0183-W06-2607150069</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr"/>
-      <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3922,14 +3566,11 @@
           <t>B0183-W06-2607150070</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr"/>
-      <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3952,14 +3593,11 @@
           <t>B0183-W06-2607150071</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr"/>
-      <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3982,14 +3620,11 @@
           <t>B0183-W06-2607150072</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr"/>
-      <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -4012,14 +3647,11 @@
           <t>B0183-W06-2607150073</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
-      <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -4042,14 +3674,11 @@
           <t>B0183-W06-2607150074</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr"/>
-      <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -4072,14 +3701,11 @@
           <t>B0183-W06-2607150075</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr"/>
-      <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -4102,14 +3728,11 @@
           <t>B0183-W06-2607150076</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr"/>
-      <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -4132,14 +3755,11 @@
           <t>B0183-W06-2607150077</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr"/>
-      <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -4162,14 +3782,11 @@
           <t>B0183-W06-2607150078</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr"/>
-      <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -4192,14 +3809,11 @@
           <t>B0183-W06-2607150079</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr"/>
-      <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -4222,14 +3836,11 @@
           <t>B0183-W06-2607150080</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr"/>
-      <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -4252,14 +3863,11 @@
           <t>B0183-W06-2607150081</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr"/>
-      <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -4282,14 +3890,11 @@
           <t>B0183-W06-2607150082</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr"/>
-      <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -4312,14 +3917,11 @@
           <t>B0183-W06-2607150083</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr"/>
-      <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -4342,14 +3944,11 @@
           <t>B0183-W06-2607150084</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr"/>
-      <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -4372,14 +3971,11 @@
           <t>B0183-W06-2607150085</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr"/>
-      <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -4402,14 +3998,11 @@
           <t>B0183-W06-2607150086</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr"/>
-      <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4432,14 +4025,11 @@
           <t>B0183-W06-2607150087</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr"/>
-      <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -4462,14 +4052,11 @@
           <t>B0183-W06-2607150088</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr"/>
-      <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -4492,14 +4079,11 @@
           <t>B0183-W06-2607150089</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr"/>
-      <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -4522,14 +4106,11 @@
           <t>B0183-W06-2607150090</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr"/>
-      <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -4552,14 +4133,11 @@
           <t>B0183-W06-2607150091</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr"/>
-      <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -4582,14 +4160,11 @@
           <t>B0183-W06-2607150092</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr"/>
-      <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -4612,14 +4187,11 @@
           <t>B0183-W06-2607150093</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr"/>
-      <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -4642,14 +4214,11 @@
           <t>B0183-W06-2607150094</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr"/>
-      <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -4672,14 +4241,11 @@
           <t>B0183-W06-2607150095</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr"/>
-      <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -4702,14 +4268,11 @@
           <t>B0183-W06-2607160001</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr"/>
-      <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -4732,14 +4295,11 @@
           <t>B0183-W06-2607160002</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr"/>
-      <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -4762,14 +4322,11 @@
           <t>B0183-W06-2607160003</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr"/>
-      <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -4792,14 +4349,11 @@
           <t>B0183-W06-2607160004</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr"/>
-      <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -4822,14 +4376,11 @@
           <t>B0183-W06-2607160005</t>
         </is>
       </c>
-      <c r="E97" t="inlineStr"/>
-      <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -4852,14 +4403,11 @@
           <t>B0183-W06-2607160006</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr"/>
-      <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -4882,14 +4430,11 @@
           <t>B0183-W06-2607160007</t>
         </is>
       </c>
-      <c r="E99" t="inlineStr"/>
-      <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -4912,14 +4457,11 @@
           <t>B0183-W06-2607160008</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr"/>
-      <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -4942,14 +4484,11 @@
           <t>B0183-W06-2607160009</t>
         </is>
       </c>
-      <c r="E101" t="inlineStr"/>
-      <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -4972,14 +4511,11 @@
           <t>B0183-W06-2607160010</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr"/>
-      <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -5002,14 +4538,11 @@
           <t>B0183-W06-2607160011</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr"/>
-      <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -5032,14 +4565,11 @@
           <t>B0183-W06-2607160012</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr"/>
-      <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -5062,14 +4592,11 @@
           <t>B0183-W06-2607160013</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr"/>
-      <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -5092,14 +4619,11 @@
           <t>B0183-W06-2607160014</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr"/>
-      <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -5122,14 +4646,11 @@
           <t>B0183-W06-2607160015</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr"/>
-      <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -5152,14 +4673,11 @@
           <t>B0183-W06-2607160016</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr"/>
-      <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -5182,14 +4700,11 @@
           <t>B0183-W06-2607160017</t>
         </is>
       </c>
-      <c r="E109" t="inlineStr"/>
-      <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -5212,14 +4727,11 @@
           <t>B0183-W06-2607160018</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr"/>
-      <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -5242,14 +4754,11 @@
           <t>B0183-W06-2607160019</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr"/>
-      <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -5272,14 +4781,11 @@
           <t>B0183-W06-2607160020</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr"/>
-      <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -5302,14 +4808,11 @@
           <t>B0183-W06-2607160021</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr"/>
-      <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -5332,14 +4835,11 @@
           <t>B0183-W06-2607160022</t>
         </is>
       </c>
-      <c r="E114" t="inlineStr"/>
-      <c r="F114" t="inlineStr"/>
       <c r="G114" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -5362,14 +4862,11 @@
           <t>B0183-W06-2607160023</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr"/>
-      <c r="F115" t="inlineStr"/>
       <c r="G115" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -5392,14 +4889,11 @@
           <t>B0183-W06-2607160024</t>
         </is>
       </c>
-      <c r="E116" t="inlineStr"/>
-      <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -5422,14 +4916,11 @@
           <t>B0183-W06-2607160025</t>
         </is>
       </c>
-      <c r="E117" t="inlineStr"/>
-      <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -5452,14 +4943,11 @@
           <t>B0183-W06-2607160026</t>
         </is>
       </c>
-      <c r="E118" t="inlineStr"/>
-      <c r="F118" t="inlineStr"/>
       <c r="G118" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -5482,14 +4970,11 @@
           <t>B0183-W06-2607160027</t>
         </is>
       </c>
-      <c r="E119" t="inlineStr"/>
-      <c r="F119" t="inlineStr"/>
       <c r="G119" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -5512,14 +4997,11 @@
           <t>B0183-W06-2607160028</t>
         </is>
       </c>
-      <c r="E120" t="inlineStr"/>
-      <c r="F120" t="inlineStr"/>
       <c r="G120" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -5542,14 +5024,11 @@
           <t>B0183-W06-2607160029</t>
         </is>
       </c>
-      <c r="E121" t="inlineStr"/>
-      <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -5572,14 +5051,11 @@
           <t>B0183-W06-2607160030</t>
         </is>
       </c>
-      <c r="E122" t="inlineStr"/>
-      <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -5602,14 +5078,11 @@
           <t>B0183-W06-2607160031</t>
         </is>
       </c>
-      <c r="E123" t="inlineStr"/>
-      <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -5632,14 +5105,11 @@
           <t>B0183-W06-2607160032</t>
         </is>
       </c>
-      <c r="E124" t="inlineStr"/>
-      <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -5662,14 +5132,11 @@
           <t>B0183-W06-2607160033</t>
         </is>
       </c>
-      <c r="E125" t="inlineStr"/>
-      <c r="F125" t="inlineStr"/>
       <c r="G125" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -5692,14 +5159,11 @@
           <t>B0183-W06-2607160034</t>
         </is>
       </c>
-      <c r="E126" t="inlineStr"/>
-      <c r="F126" t="inlineStr"/>
       <c r="G126" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -5722,14 +5186,11 @@
           <t>B0183-W06-2607160035</t>
         </is>
       </c>
-      <c r="E127" t="inlineStr"/>
-      <c r="F127" t="inlineStr"/>
       <c r="G127" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -5752,14 +5213,11 @@
           <t>B0183-W06-2607160036</t>
         </is>
       </c>
-      <c r="E128" t="inlineStr"/>
-      <c r="F128" t="inlineStr"/>
       <c r="G128" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -5782,14 +5240,11 @@
           <t>B0183-W06-2607160037</t>
         </is>
       </c>
-      <c r="E129" t="inlineStr"/>
-      <c r="F129" t="inlineStr"/>
       <c r="G129" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -5812,14 +5267,11 @@
           <t>B0183-W06-2607160038</t>
         </is>
       </c>
-      <c r="E130" t="inlineStr"/>
-      <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -5842,14 +5294,11 @@
           <t>B0183-W06-2607160039</t>
         </is>
       </c>
-      <c r="E131" t="inlineStr"/>
-      <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -5872,14 +5321,11 @@
           <t>B0183-W06-2607160040</t>
         </is>
       </c>
-      <c r="E132" t="inlineStr"/>
-      <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -5902,14 +5348,11 @@
           <t>B0183-W06-2607160041</t>
         </is>
       </c>
-      <c r="E133" t="inlineStr"/>
-      <c r="F133" t="inlineStr"/>
       <c r="G133" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -5932,14 +5375,11 @@
           <t>B0183-W06-2607160042</t>
         </is>
       </c>
-      <c r="E134" t="inlineStr"/>
-      <c r="F134" t="inlineStr"/>
       <c r="G134" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -5962,14 +5402,11 @@
           <t>B0183-W06-2607160043</t>
         </is>
       </c>
-      <c r="E135" t="inlineStr"/>
-      <c r="F135" t="inlineStr"/>
       <c r="G135" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -5992,14 +5429,11 @@
           <t>B0183-W06-2607160044</t>
         </is>
       </c>
-      <c r="E136" t="inlineStr"/>
-      <c r="F136" t="inlineStr"/>
       <c r="G136" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -6022,14 +5456,11 @@
           <t>B0183-W06-2607160045</t>
         </is>
       </c>
-      <c r="E137" t="inlineStr"/>
-      <c r="F137" t="inlineStr"/>
       <c r="G137" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -6052,14 +5483,11 @@
           <t>B0183-W06-2607160046</t>
         </is>
       </c>
-      <c r="E138" t="inlineStr"/>
-      <c r="F138" t="inlineStr"/>
       <c r="G138" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -6082,14 +5510,11 @@
           <t>B0183-W06-2607160047</t>
         </is>
       </c>
-      <c r="E139" t="inlineStr"/>
-      <c r="F139" t="inlineStr"/>
       <c r="G139" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -6112,14 +5537,11 @@
           <t>B0183-W06-2607160048</t>
         </is>
       </c>
-      <c r="E140" t="inlineStr"/>
-      <c r="F140" t="inlineStr"/>
       <c r="G140" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -6142,14 +5564,11 @@
           <t>B0183-W06-2607160049</t>
         </is>
       </c>
-      <c r="E141" t="inlineStr"/>
-      <c r="F141" t="inlineStr"/>
       <c r="G141" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -6172,14 +5591,11 @@
           <t>B0183-W06-2607160050</t>
         </is>
       </c>
-      <c r="E142" t="inlineStr"/>
-      <c r="F142" t="inlineStr"/>
       <c r="G142" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -6202,14 +5618,11 @@
           <t>B0183-W06-2607160051</t>
         </is>
       </c>
-      <c r="E143" t="inlineStr"/>
-      <c r="F143" t="inlineStr"/>
       <c r="G143" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -6232,14 +5645,11 @@
           <t>B0183-W06-2607160052</t>
         </is>
       </c>
-      <c r="E144" t="inlineStr"/>
-      <c r="F144" t="inlineStr"/>
       <c r="G144" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -6262,14 +5672,11 @@
           <t>B0183-W06-2607160053</t>
         </is>
       </c>
-      <c r="E145" t="inlineStr"/>
-      <c r="F145" t="inlineStr"/>
       <c r="G145" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -6292,14 +5699,11 @@
           <t>B0183-W06-2607160054</t>
         </is>
       </c>
-      <c r="E146" t="inlineStr"/>
-      <c r="F146" t="inlineStr"/>
       <c r="G146" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -6322,14 +5726,11 @@
           <t>B0183-W06-2607160055</t>
         </is>
       </c>
-      <c r="E147" t="inlineStr"/>
-      <c r="F147" t="inlineStr"/>
       <c r="G147" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -6352,14 +5753,11 @@
           <t>B0183-W06-2607160056</t>
         </is>
       </c>
-      <c r="E148" t="inlineStr"/>
-      <c r="F148" t="inlineStr"/>
       <c r="G148" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -6382,14 +5780,11 @@
           <t>B0183-W06-2607160057</t>
         </is>
       </c>
-      <c r="E149" t="inlineStr"/>
-      <c r="F149" t="inlineStr"/>
       <c r="G149" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -6412,14 +5807,11 @@
           <t>B0183-W06-2607160058</t>
         </is>
       </c>
-      <c r="E150" t="inlineStr"/>
-      <c r="F150" t="inlineStr"/>
       <c r="G150" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -6442,14 +5834,11 @@
           <t>B0183-W06-2607160059</t>
         </is>
       </c>
-      <c r="E151" t="inlineStr"/>
-      <c r="F151" t="inlineStr"/>
       <c r="G151" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -6472,14 +5861,11 @@
           <t>B0183-W06-2607160060</t>
         </is>
       </c>
-      <c r="E152" t="inlineStr"/>
-      <c r="F152" t="inlineStr"/>
       <c r="G152" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -6502,14 +5888,11 @@
           <t>B0183-W06-2607160061</t>
         </is>
       </c>
-      <c r="E153" t="inlineStr"/>
-      <c r="F153" t="inlineStr"/>
       <c r="G153" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -6532,14 +5915,11 @@
           <t>B0183-W06-2607160062</t>
         </is>
       </c>
-      <c r="E154" t="inlineStr"/>
-      <c r="F154" t="inlineStr"/>
       <c r="G154" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -6562,14 +5942,11 @@
           <t>B0183-W06-2607160063</t>
         </is>
       </c>
-      <c r="E155" t="inlineStr"/>
-      <c r="F155" t="inlineStr"/>
       <c r="G155" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -6592,14 +5969,11 @@
           <t>B0183-W06-2607160064</t>
         </is>
       </c>
-      <c r="E156" t="inlineStr"/>
-      <c r="F156" t="inlineStr"/>
       <c r="G156" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -6622,14 +5996,11 @@
           <t>B0183-W06-2607160065</t>
         </is>
       </c>
-      <c r="E157" t="inlineStr"/>
-      <c r="F157" t="inlineStr"/>
       <c r="G157" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -6652,14 +6023,11 @@
           <t>B0183-W06-2607160066</t>
         </is>
       </c>
-      <c r="E158" t="inlineStr"/>
-      <c r="F158" t="inlineStr"/>
       <c r="G158" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -6682,14 +6050,11 @@
           <t>B0183-W06-2607160067</t>
         </is>
       </c>
-      <c r="E159" t="inlineStr"/>
-      <c r="F159" t="inlineStr"/>
       <c r="G159" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="H159" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6733,7 +6098,6 @@
           <t>260714ME2SPR8B</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -6746,7 +6110,6 @@
           <t>260714MAABXFNA</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -6759,7 +6122,6 @@
           <t>260714MFH9DW2A</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -6772,7 +6134,6 @@
           <t>260714M73X4KDD</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -6785,7 +6146,6 @@
           <t>260714N804HATB</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -6798,7 +6158,6 @@
           <t>260714NE90AT6Q</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -6811,7 +6170,6 @@
           <t>260715NS3JMKN4</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -6824,7 +6182,6 @@
           <t>260715P8GEFXQA</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -6837,7 +6194,6 @@
           <t>260715NSQ8YY0M</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -6850,7 +6206,6 @@
           <t>260714MG4W0FE1</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -6863,7 +6218,6 @@
           <t>260714MGDCSTKD</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -6876,7 +6230,6 @@
           <t>260714MSB2NRHW</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -6889,7 +6242,6 @@
           <t>260714MTQNE9KH</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -6902,7 +6254,6 @@
           <t>260714NDJK69K6</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -6915,7 +6266,6 @@
           <t>260715NN0ANF8M</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -6928,7 +6278,6 @@
           <t>260715NRN7XHMQ</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -6941,7 +6290,6 @@
           <t>260715NTW9WGVX</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -6954,7 +6302,6 @@
           <t>260715P8NW0089</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -6967,7 +6314,6 @@
           <t>260715P2TECXYE</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -6980,7 +6326,6 @@
           <t>260714MEQXT9JG</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -6993,7 +6338,6 @@
           <t>260714MERJURDH</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -7006,7 +6350,6 @@
           <t>260714NACRFQJD</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -7019,7 +6362,6 @@
           <t>260714NB1DAW1V</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -7032,7 +6374,6 @@
           <t>260715PFJNV558</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -7045,7 +6386,6 @@
           <t>260714NGFC0C1K</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -7058,7 +6398,6 @@
           <t>260714NM0XCJQE</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -7071,7 +6410,6 @@
           <t>260715NSJFGCXY</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -7084,7 +6422,6 @@
           <t>260715PHRBHNR0</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -7097,7 +6434,6 @@
           <t>260714NJCRGNVB</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -7110,7 +6446,6 @@
           <t>260715NWP2UAYJ</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -7118,8 +6453,6 @@
           <t>260714MYVJ3YKY</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr"/>
-      <c r="C32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -7127,8 +6460,6 @@
           <t>260714NGFC0C1K</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr"/>
-      <c r="C33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -7136,8 +6467,6 @@
           <t>260714NM0XCJQE</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr"/>
-      <c r="C34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -7145,8 +6474,6 @@
           <t>260715NSJFGCXY</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr"/>
-      <c r="C35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -7154,8 +6481,6 @@
           <t>260715PHRBHNR0</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr"/>
-      <c r="C36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -7163,8 +6488,6 @@
           <t>260714N8XQ0K9D</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr"/>
-      <c r="C37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -7172,8 +6495,6 @@
           <t>260715NPU39T1A</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr"/>
-      <c r="C38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -7181,8 +6502,6 @@
           <t>260714NJCRGNVB</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr"/>
-      <c r="C39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -7190,8 +6509,6 @@
           <t>260715NWP2UAYJ</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr"/>
-      <c r="C40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -7199,8 +6516,6 @@
           <t>260715NRKNBJR8</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr"/>
-      <c r="C41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -7208,8 +6523,6 @@
           <t>260714MGE2NRAR</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr"/>
-      <c r="C42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -7217,8 +6530,6 @@
           <t>260714MRY9Y24A</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr"/>
-      <c r="C43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -7226,8 +6537,6 @@
           <t>260714NAWP431Y</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr"/>
-      <c r="C44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -7235,8 +6544,6 @@
           <t>260714NE3RG27F</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr"/>
-      <c r="C45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -7244,8 +6551,6 @@
           <t>260715NQ636K6M</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr"/>
-      <c r="C46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -7253,8 +6558,6 @@
           <t>260715PK02QM5W</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr"/>
-      <c r="C47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -7262,8 +6565,6 @@
           <t>260715PH3UCNRG</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr"/>
-      <c r="C48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -7271,8 +6572,6 @@
           <t>260715PMS8WJS4</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr"/>
-      <c r="C49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -7280,8 +6579,6 @@
           <t>260715PN1TJV6C</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr"/>
-      <c r="C50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -7289,8 +6586,6 @@
           <t>260715NTN1NU8C</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr"/>
-      <c r="C51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -7298,8 +6593,6 @@
           <t>260714M4W8YWJM</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr"/>
-      <c r="C52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -7307,8 +6600,6 @@
           <t>260714NJT9FHW1</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr"/>
-      <c r="C53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -7316,8 +6607,6 @@
           <t>260715NS752BR6</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr"/>
-      <c r="C54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -7325,8 +6614,6 @@
           <t>260714MVE1VSM3</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr"/>
-      <c r="C55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -7334,8 +6621,6 @@
           <t>260714N2H4MSE7</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr"/>
-      <c r="C56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -7343,8 +6628,6 @@
           <t>260715PERYSRUS</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr"/>
-      <c r="C57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -7352,8 +6635,6 @@
           <t>260715PHRJ6APD</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr"/>
-      <c r="C58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -7361,8 +6642,6 @@
           <t>260714NDRHX0X1</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr"/>
-      <c r="C59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -7370,8 +6649,6 @@
           <t>260714MX1KP61B</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr"/>
-      <c r="C60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -7379,8 +6656,6 @@
           <t>260715NRFHPUX5</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr"/>
-      <c r="C61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -7388,8 +6663,6 @@
           <t>260714MR0GU8WT</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr"/>
-      <c r="C62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -7397,8 +6670,6 @@
           <t>260714NCQ5U9U4</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr"/>
-      <c r="C63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -7406,8 +6677,6 @@
           <t>260714NEFXGYVK</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr"/>
-      <c r="C64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -7415,8 +6684,6 @@
           <t>260715NRF2ERRB</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr"/>
-      <c r="C65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -7424,8 +6691,6 @@
           <t>260714NDK5B1BC</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr"/>
-      <c r="C66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -7433,8 +6698,6 @@
           <t>260715P4XAUP8H</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr"/>
-      <c r="C67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -7442,8 +6705,6 @@
           <t>260715PHRSUDUV</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr"/>
-      <c r="C68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -7451,8 +6712,6 @@
           <t>260714MPHSFJYJ</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr"/>
-      <c r="C69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -7460,8 +6719,6 @@
           <t>260714NJN5F1YC</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr"/>
-      <c r="C70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -7469,8 +6726,6 @@
           <t>260715NRHJMG8M</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr"/>
-      <c r="C71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -7478,8 +6733,6 @@
           <t>260715PDEQEJ6U</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr"/>
-      <c r="C72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -7487,8 +6740,6 @@
           <t>260714MW6TCMBV</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr"/>
-      <c r="C73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -7496,8 +6747,6 @@
           <t>260715PPM5AGCE</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr"/>
-      <c r="C74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -7505,8 +6754,6 @@
           <t>260714MSW9BFJC</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr"/>
-      <c r="C75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -7514,8 +6761,6 @@
           <t>260714MV7NR6WM</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr"/>
-      <c r="C76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -7523,8 +6768,6 @@
           <t>260714N9U7PX1R</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr"/>
-      <c r="C77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -7532,8 +6775,6 @@
           <t>260714NCF83NFG</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr"/>
-      <c r="C78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -7541,8 +6782,6 @@
           <t>260715P1E1EY72</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr"/>
-      <c r="C79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -7550,8 +6789,6 @@
           <t>260714N8BHU8K8</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr"/>
-      <c r="C80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -7559,8 +6796,6 @@
           <t>260714MKJU4987</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr"/>
-      <c r="C81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -7568,8 +6803,6 @@
           <t>260715NNY8HRCB</t>
         </is>
       </c>
-      <c r="B82" t="inlineStr"/>
-      <c r="C82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -7577,8 +6810,6 @@
           <t>260715NNNSAE9D</t>
         </is>
       </c>
-      <c r="B83" t="inlineStr"/>
-      <c r="C83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -7586,8 +6817,6 @@
           <t>260714K7FNP2QN</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr"/>
-      <c r="C84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -7595,8 +6824,6 @@
           <t>260714NBJU8C39</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr"/>
-      <c r="C85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -7604,8 +6831,6 @@
           <t>260715NYNUSPAY</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr"/>
-      <c r="C86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -7613,8 +6838,6 @@
           <t>260714NFMBY4MG</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr"/>
-      <c r="C87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -7622,8 +6845,6 @@
           <t>260715NUA5WBDC</t>
         </is>
       </c>
-      <c r="B88" t="inlineStr"/>
-      <c r="C88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -7631,8 +6852,6 @@
           <t>260715NP5QF71C</t>
         </is>
       </c>
-      <c r="B89" t="inlineStr"/>
-      <c r="C89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -7640,8 +6859,6 @@
           <t>260714NCBPMEV1</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr"/>
-      <c r="C90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -7649,8 +6866,6 @@
           <t>260715NW0APK8H</t>
         </is>
       </c>
-      <c r="B91" t="inlineStr"/>
-      <c r="C91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -7658,8 +6873,6 @@
           <t>260714MQTF8GRE</t>
         </is>
       </c>
-      <c r="B92" t="inlineStr"/>
-      <c r="C92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -7667,8 +6880,6 @@
           <t>260714N3XRPAKE</t>
         </is>
       </c>
-      <c r="B93" t="inlineStr"/>
-      <c r="C93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -7676,8 +6887,6 @@
           <t>260714MB47PS0A</t>
         </is>
       </c>
-      <c r="B94" t="inlineStr"/>
-      <c r="C94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -7685,8 +6894,6 @@
           <t>260715NUQ4QEDK</t>
         </is>
       </c>
-      <c r="B95" t="inlineStr"/>
-      <c r="C95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -7694,8 +6901,6 @@
           <t>260715PKCP4YWJ</t>
         </is>
       </c>
-      <c r="B96" t="inlineStr"/>
-      <c r="C96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -7703,8 +6908,6 @@
           <t>260714MQJ8YM2Q</t>
         </is>
       </c>
-      <c r="B97" t="inlineStr"/>
-      <c r="C97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -7712,8 +6915,6 @@
           <t>260715NUM77VPM</t>
         </is>
       </c>
-      <c r="B98" t="inlineStr"/>
-      <c r="C98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -7721,8 +6922,6 @@
           <t>260714MAP8FUBW</t>
         </is>
       </c>
-      <c r="B99" t="inlineStr"/>
-      <c r="C99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -7730,8 +6929,6 @@
           <t>260714MFCFWP3R</t>
         </is>
       </c>
-      <c r="B100" t="inlineStr"/>
-      <c r="C100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -7739,8 +6936,6 @@
           <t>260715NRDKRPCB</t>
         </is>
       </c>
-      <c r="B101" t="inlineStr"/>
-      <c r="C101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -7748,8 +6943,6 @@
           <t>260714NGG9G8Q8</t>
         </is>
       </c>
-      <c r="B102" t="inlineStr"/>
-      <c r="C102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -7757,8 +6950,67 @@
           <t>260714KAPC1CN2</t>
         </is>
       </c>
-      <c r="B103" t="inlineStr"/>
-      <c r="C103" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>timestamp</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>tracking</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>orders</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>bill_no</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>price</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>sn</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>error_category</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>remark</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>